<commit_message>
v8.0 complete: full check PASS (section 14 rule for stable names); old method notes removed (Methods chapters in docs/methods/), references point to the chapters; Excel review checklist in plans/; documents regenerated; CAVEATS entry
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TEE6PTp5h76eJpJAS6na67
</commit_message>
<xml_diff>
--- a/excel_ai/CPAT-AI_BugsAndIssues_latest.xlsx
+++ b/excel_ai/CPAT-AI_BugsAndIssues_latest.xlsx
@@ -1656,7 +1656,7 @@
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>Taxes jump in the first projected year when pass-through is between 0 and 1 (none for Egypt: 0 or 1). prototype: Fixed in v4.10 (user rule: bugs are never replicated): the floating part is (1 - pass-through) x (last tax + fall in supply cost), applied once (txf; PriceProjection_Method.md A10); no effect for Egypt (pass-through 0 or 1).</t>
+          <t>Taxes jump in the first projected year when pass-through is between 0 and 1 (none for Egypt: 0 or 1). prototype: Fixed in v4.10 (user rule: bugs are never replicated): the floating part is (1 - pass-through) x (last tax + fall in supply cost), applied once (txf; Methods, chapter Prices A10); no effect for Egypt (pass-through 0 or 1).</t>
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>Non-energy methane is flat and a methane fee on agriculture and waste has no effect. prototype: Fixed in v2.8: the sources grow with income and population and the fee abates them along their curves (GHG_Method.md).</t>
+          <t>Non-energy methane is flat and a methane fee on agriculture and waste has no effect. prototype: Fixed in v2.8: the sources grow with income and population and the fee abates them along their curves (Methods, chapter Emissions).</t>
         </is>
       </c>
       <c r="I20" s="9" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I27" s="9" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
-          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I28" s="9" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>Egypt engineer baseline 2035: gasoline -33.9%, diesel -37.9%, road electricity -52.4%, passenger EV sales share -2.6 points. prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>Egypt engineer baseline 2035: gasoline -33.9%, diesel -37.9%, road electricity -52.4%, passenger EV sales share -2.6 points. prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I29" s="9" t="inlineStr">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t>Egypt engineer baseline 2035: gasoline +0.0%, diesel +0.0%, road electricity -0.6%, passenger EV sales share -0.1 points. prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>Egypt engineer baseline 2035: gasoline +0.0%, diesel +0.0%, road electricity -0.6%, passenger EV sales share -0.1 points. prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I30" s="9" t="inlineStr">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I31" s="9" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="H32" s="9" t="inlineStr">
         <is>
-          <t>Egypt engineer baseline 2035: gasoline +0.0%, diesel -0.3%, road electricity -16.8%, passenger EV sales share +0.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>Egypt engineer baseline 2035: gasoline +0.0%, diesel -0.3%, road electricity -16.8%, passenger EV sales share +0.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I32" s="9" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>Egypt engineer baseline 2035: gasoline -0.0%, diesel +0.0%, road electricity -0.3%, passenger EV sales share +0.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>Egypt engineer baseline 2035: gasoline -0.0%, diesel +0.0%, road electricity -0.3%, passenger EV sales share +0.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I33" s="9" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
-          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I34" s="9" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="H35" s="9" t="inlineStr">
         <is>
-          <t>Egypt engineer baseline 2035: gasoline -0.0%, diesel -0.2%, road electricity +4.0%, passenger EV sales share +0.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>Egypt engineer baseline 2035: gasoline -0.0%, diesel -0.2%, road electricity +4.0%, passenger EV sales share +0.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I35" s="9" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="H36" s="9" t="inlineStr">
         <is>
-          <t>Egypt engineer baseline 2035: gasoline +0.0%, diesel +0.2%, road electricity -1.0%, passenger EV sales share -0.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>Egypt engineer baseline 2035: gasoline +0.0%, diesel +0.2%, road electricity -1.0%, passenger EV sales share -0.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I36" s="9" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
-          <t>Egypt engineer baseline 2035: gasoline -0.0%, diesel +0.1%, road electricity +0.2%, passenger EV sales share +0.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>Egypt engineer baseline 2035: gasoline -0.0%, diesel +0.1%, road electricity +0.2%, passenger EV sales share +0.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I37" s="9" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="H38" s="9" t="inlineStr">
         <is>
-          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I38" s="9" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="H39" s="9" t="inlineStr">
         <is>
-          <t>Egypt engineer baseline 2035: gasoline -0.1%, diesel -0.0%, road electricity +1.2%, passenger EV sales share +0.5 points. prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>Egypt engineer baseline 2035: gasoline -0.1%, diesel -0.0%, road electricity +1.2%, passenger EV sales share +0.5 points. prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I39" s="9" t="inlineStr">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="H40" s="9" t="inlineStr">
         <is>
-          <t>Egypt engineer baseline 2035: gasoline +5.1%, diesel +3.1%, road electricity -50.7%, passenger EV sales share -10.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>Egypt engineer baseline 2035: gasoline +5.1%, diesel +3.1%, road electricity -50.7%, passenger EV sales share -10.0 points. prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I40" s="9" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I41" s="9" t="inlineStr">
@@ -3081,7 +3081,7 @@
       </c>
       <c r="H42" s="9" t="inlineStr">
         <is>
-          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I42" s="9" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="H43" s="9" t="inlineStr">
         <is>
-          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Transport_vs_Legacy.md); latent in the legacy Egypt run (elasticity road model).</t>
+          <t>None in the Egypt engineer run (the policy or fuel is zero there). prototype: Fixed in the prototype engineer road model (v3.5; Methods, chapter Transport); latent in the legacy Egypt run (elasticity road model).</t>
         </is>
       </c>
       <c r="I43" s="9" t="inlineStr">
@@ -8388,7 +8388,7 @@
       </c>
       <c r="J135" s="9" t="inlineStr">
         <is>
-          <t>PowerPrices_Method.md 3.9</t>
+          <t>Methods, chapter Power 3.9</t>
         </is>
       </c>
       <c r="K135" s="9" t="inlineStr">
@@ -8494,7 +8494,7 @@
       </c>
       <c r="J137" s="9" t="inlineStr">
         <is>
-          <t>PowerPrices_Method.md; LegacyDiff</t>
+          <t>Methods, chapter Power; LegacyDiff</t>
         </is>
       </c>
       <c r="K137" s="9" t="inlineStr">
@@ -8547,7 +8547,7 @@
       </c>
       <c r="J138" s="9" t="inlineStr">
         <is>
-          <t>GDP_Method.md; LegacyDiff 55</t>
+          <t>Methods, chapter Macro and results; LegacyDiff 55</t>
         </is>
       </c>
       <c r="K138" s="9" t="inlineStr">
@@ -8706,7 +8706,7 @@
       </c>
       <c r="J141" s="9" t="inlineStr">
         <is>
-          <t>PowerPrices_Method.md; LegacyDiff 77</t>
+          <t>Methods, chapter Power; LegacyDiff 77</t>
         </is>
       </c>
       <c r="K141" s="9" t="inlineStr">
@@ -8759,7 +8759,7 @@
       </c>
       <c r="J142" s="9" t="inlineStr">
         <is>
-          <t>GHG_Method.md; LegacyDiff</t>
+          <t>Methods, chapter Emissions; LegacyDiff</t>
         </is>
       </c>
       <c r="K142" s="9" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="J143" s="9" t="inlineStr">
         <is>
-          <t>PriceProjection_Method.md; LegacyDiff</t>
+          <t>Methods, chapter Prices; LegacyDiff</t>
         </is>
       </c>
       <c r="K143" s="9" t="inlineStr">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="J144" s="9" t="inlineStr">
         <is>
-          <t>GHG_Method.md</t>
+          <t>Methods, chapter Emissions</t>
         </is>
       </c>
       <c r="K144" s="9" t="inlineStr">
@@ -8918,7 +8918,7 @@
       </c>
       <c r="J145" s="9" t="inlineStr">
         <is>
-          <t>Plans.md (section Plan_AirPollution)</t>
+          <t>excel_ai/plans/Air_pollution.md</t>
         </is>
       </c>
       <c r="K145" s="9" t="inlineStr">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="J146" s="9" t="inlineStr">
         <is>
-          <t>Plans.md (section Plan_TransportExternalities)</t>
+          <t>excel_ai/plans/Transport_cobenefits.md</t>
         </is>
       </c>
       <c r="K146" s="9" t="inlineStr">
@@ -9077,7 +9077,7 @@
       </c>
       <c r="J148" s="9" t="inlineStr">
         <is>
-          <t>legacy_comparison_v6_4.md; PriceProjection_Method.md A7</t>
+          <t>legacy_comparison_v6_4.md; Methods, chapter Prices A7</t>
         </is>
       </c>
       <c r="K148" s="9" t="inlineStr">
@@ -9130,7 +9130,7 @@
       </c>
       <c r="J149" s="9" t="inlineStr">
         <is>
-          <t>GHG_Method.md (Data); CAVEATS v2.8</t>
+          <t>Methods, chapter Emissions (Data); CAVEATS v2.8</t>
         </is>
       </c>
       <c r="K149" s="9" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="J150" s="9" t="inlineStr">
         <is>
-          <t>CO2Calibration_Method.md; CAVEATS v3.2</t>
+          <t>Methods, chapter Emissions; CAVEATS v3.2</t>
         </is>
       </c>
       <c r="K150" s="9" t="inlineStr">
@@ -9289,7 +9289,7 @@
       </c>
       <c r="J152" s="9" t="inlineStr">
         <is>
-          <t>ETS_Method.md; ETS_Legacy_Algorithm.md; LegacyDiff</t>
+          <t>Methods, chapter ETS; Methods, chapter ETS; LegacyDiff</t>
         </is>
       </c>
       <c r="K152" s="9" t="inlineStr">
@@ -9448,7 +9448,7 @@
       </c>
       <c r="J155" s="9" t="inlineStr">
         <is>
-          <t>GHG_Method.md; CAVEATS v2.8</t>
+          <t>Methods, chapter Emissions; CAVEATS v2.8</t>
         </is>
       </c>
       <c r="K155" s="9" t="inlineStr">
@@ -9501,7 +9501,7 @@
       </c>
       <c r="J156" s="9" t="inlineStr">
         <is>
-          <t>Transport_vs_Legacy.md</t>
+          <t>Methods, chapter Transport</t>
         </is>
       </c>
       <c r="K156" s="9" t="inlineStr">
@@ -9607,7 +9607,7 @@
       </c>
       <c r="J158" s="9" t="inlineStr">
         <is>
-          <t>ResultsSections_Method.md; CO2Calibration_Method.md; CAVEATS v4.11</t>
+          <t>Methods, chapter Macro and results; Methods, chapter Emissions; CAVEATS v4.11</t>
         </is>
       </c>
       <c r="K158" s="9" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="J159" s="9" t="inlineStr">
         <is>
-          <t>AirPollutants_Method.md; CAVEATS v3.12</t>
+          <t>Methods, chapter Emissions; CAVEATS v3.12</t>
         </is>
       </c>
       <c r="K159" s="9" t="inlineStr">
@@ -9713,7 +9713,7 @@
       </c>
       <c r="J160" s="9" t="inlineStr">
         <is>
-          <t>ResultsSections_Method.md; CAVEATS v3.15</t>
+          <t>Methods, chapter Macro and results; CAVEATS v3.15</t>
         </is>
       </c>
       <c r="K160" s="9" t="inlineStr">
@@ -9766,7 +9766,7 @@
       </c>
       <c r="J161" s="9" t="inlineStr">
         <is>
-          <t>ResultsSections_Method.md</t>
+          <t>Methods, chapter Macro and results</t>
         </is>
       </c>
       <c r="K161" s="9" t="inlineStr">
@@ -9819,7 +9819,7 @@
       </c>
       <c r="J162" s="9" t="inlineStr">
         <is>
-          <t>DataTabs.md; CAVEATS v4.7</t>
+          <t>Methods, chapter Data tabs; CAVEATS v4.7</t>
         </is>
       </c>
       <c r="K162" s="9" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J163" s="9" t="inlineStr">
         <is>
-          <t>PriceProjection_Method.md 5; LegacyDiff</t>
+          <t>Methods, chapter Prices 5; LegacyDiff</t>
         </is>
       </c>
       <c r="K163" s="9" t="inlineStr">
@@ -9925,7 +9925,7 @@
       </c>
       <c r="J164" s="9" t="inlineStr">
         <is>
-          <t>Transport_Method.md; LegacyDiff</t>
+          <t>Methods, chapter Transport; LegacyDiff</t>
         </is>
       </c>
       <c r="K164" s="9" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="J165" s="9" t="inlineStr">
         <is>
-          <t>GDP_Method.md; LegacyDiff</t>
+          <t>Methods, chapter Macro and results; LegacyDiff</t>
         </is>
       </c>
       <c r="K165" s="9" t="inlineStr">
@@ -10031,7 +10031,7 @@
       </c>
       <c r="J166" s="9" t="inlineStr">
         <is>
-          <t>GDP_Method.md</t>
+          <t>Methods, chapter Macro and results</t>
         </is>
       </c>
       <c r="K166" s="9" t="inlineStr">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="J167" s="9" t="inlineStr">
         <is>
-          <t>GDP_Method.md</t>
+          <t>Methods, chapter Macro and results</t>
         </is>
       </c>
       <c r="K167" s="9" t="inlineStr">
@@ -10137,7 +10137,7 @@
       </c>
       <c r="J168" s="9" t="inlineStr">
         <is>
-          <t>GDP_Method.md</t>
+          <t>Methods, chapter Macro and results</t>
         </is>
       </c>
       <c r="K168" s="9" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="J169" s="9" t="inlineStr">
         <is>
-          <t>GDP_Method.md</t>
+          <t>Methods, chapter Macro and results</t>
         </is>
       </c>
       <c r="K169" s="9" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="J171" s="9" t="inlineStr">
         <is>
-          <t>PriceProjection_Method.md 6</t>
+          <t>Methods, chapter Prices 6</t>
         </is>
       </c>
       <c r="K171" s="9" t="inlineStr">
@@ -10349,7 +10349,7 @@
       </c>
       <c r="J172" s="9" t="inlineStr">
         <is>
-          <t>PriceProjection_Method.md 6</t>
+          <t>Methods, chapter Prices 6</t>
         </is>
       </c>
       <c r="K172" s="9" t="inlineStr">
@@ -10402,7 +10402,7 @@
       </c>
       <c r="J173" s="9" t="inlineStr">
         <is>
-          <t>PriceProjection_Method.md 5; LegacyDiff 66</t>
+          <t>Methods, chapter Prices 5; LegacyDiff 66</t>
         </is>
       </c>
       <c r="K173" s="9" t="inlineStr">
@@ -10508,7 +10508,7 @@
       </c>
       <c r="J175" s="9" t="inlineStr">
         <is>
-          <t>PowerModel_Method.md; LegacyDiff 75</t>
+          <t>Methods, chapter Power; LegacyDiff 75</t>
         </is>
       </c>
       <c r="K175" s="9" t="inlineStr">
@@ -10561,7 +10561,7 @@
       </c>
       <c r="J176" s="9" t="inlineStr">
         <is>
-          <t>PowerPrices_Method.md; LegacyDiff 76</t>
+          <t>Methods, chapter Power; LegacyDiff 76</t>
         </is>
       </c>
       <c r="K176" s="9" t="inlineStr">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="J177" s="9" t="inlineStr">
         <is>
-          <t>PowerPrices_Method.md; LegacyDiff 77</t>
+          <t>Methods, chapter Power; LegacyDiff 77</t>
         </is>
       </c>
       <c r="K177" s="9" t="inlineStr">
@@ -10667,7 +10667,7 @@
       </c>
       <c r="J178" s="9" t="inlineStr">
         <is>
-          <t>PowerModel_Method.md; LegacyDiff 78</t>
+          <t>Methods, chapter Power; LegacyDiff 78</t>
         </is>
       </c>
       <c r="K178" s="9" t="inlineStr">
@@ -10720,7 +10720,7 @@
       </c>
       <c r="J179" s="9" t="inlineStr">
         <is>
-          <t>PowerPrices_Method.md</t>
+          <t>Methods, chapter Power</t>
         </is>
       </c>
       <c r="K179" s="9" t="inlineStr">
@@ -10773,7 +10773,7 @@
       </c>
       <c r="J180" s="9" t="inlineStr">
         <is>
-          <t>PowerPrices_Method.md</t>
+          <t>Methods, chapter Power</t>
         </is>
       </c>
       <c r="K180" s="9" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="J181" s="9" t="inlineStr">
         <is>
-          <t>Transport_Method.md; TODO</t>
+          <t>Methods, chapter Transport; TODO</t>
         </is>
       </c>
       <c r="K181" s="9" t="inlineStr">
@@ -10879,7 +10879,7 @@
       </c>
       <c r="J182" s="9" t="inlineStr">
         <is>
-          <t>PriceProjection_Method.md; TODO</t>
+          <t>Methods, chapter Prices; TODO</t>
         </is>
       </c>
       <c r="K182" s="9" t="inlineStr">
@@ -10932,7 +10932,7 @@
       </c>
       <c r="J183" s="9" t="inlineStr">
         <is>
-          <t>PriceProjection_Method.md; TODO</t>
+          <t>Methods, chapter Prices; TODO</t>
         </is>
       </c>
       <c r="K183" s="9" t="inlineStr">
@@ -10985,7 +10985,7 @@
       </c>
       <c r="J184" s="9" t="inlineStr">
         <is>
-          <t>GHG_Method.md</t>
+          <t>Methods, chapter Emissions</t>
         </is>
       </c>
       <c r="K184" s="9" t="inlineStr">
@@ -11038,7 +11038,7 @@
       </c>
       <c r="J185" s="9" t="inlineStr">
         <is>
-          <t>GHG_Method.md</t>
+          <t>Methods, chapter Emissions</t>
         </is>
       </c>
       <c r="K185" s="9" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="J186" s="9" t="inlineStr">
         <is>
-          <t>Equations.md E53-E56; PriceProjection_Method.md</t>
+          <t>Equations.md E53-E56; Methods, chapter Prices</t>
         </is>
       </c>
       <c r="K186" s="9" t="inlineStr">
@@ -11139,12 +11139,12 @@
       <c r="H187" s="9" t="inlineStr"/>
       <c r="I187" s="9" t="inlineStr">
         <is>
-          <t>Stated as a rule (user 2026-10-20): GDP_Method.md section Timing rule and NORMS (circular references): revenue of year t moves GDP only from year t+1, the fiscal space reads revenue of year t only, and no same-year GDP effect reaches same-year demand. Recommendation to the CPAT team: state it in the legacy method too.</t>
+          <t>Stated as a rule (user 2026-10-20): Methods, chapter Macro and results section Timing rule and NORMS (circular references): revenue of year t moves GDP only from year t+1, the fiscal space reads revenue of year t only, and no same-year GDP effect reaches same-year demand. Recommendation to the CPAT team: state it in the legacy method too.</t>
         </is>
       </c>
       <c r="J187" s="9" t="inlineStr">
         <is>
-          <t>GDP_Method.md; NORMS (circular references)</t>
+          <t>Methods, chapter Macro and results; NORMS (circular references)</t>
         </is>
       </c>
       <c r="K187" s="9" t="inlineStr">
@@ -11965,7 +11965,7 @@
       </c>
       <c r="F204" s="9" t="inlineStr">
         <is>
-          <t>Departs from legacy: Section 5b of every scenario group, every row live (Transport_Workbook_Notes.md); TrModel default Elasticity, Engineer by switch; the 17 legacy bugs of Transport_vs_Legacy.md section 3 fixed (B1-B23)</t>
+          <t>Departs from legacy: Section 5b of every scenario group, every row live (Methods, chapter Transport); TrModel default Elasticity, Engineer by switch; the 17 legacy bugs of Methods, chapter Transport section 3 fixed (B1-B23)</t>
         </is>
       </c>
       <c r="G204" s="9" t="inlineStr">
@@ -11975,7 +11975,7 @@
       </c>
       <c r="H204" s="9" t="inlineStr">
         <is>
-          <t>None by default; with Engineer: road fuel use and EV shares as in Transport_vs_Legacy.md section 4</t>
+          <t>None by default; with Engineer: road fuel use and EV shares as in Methods, chapter Transport section 4</t>
         </is>
       </c>
       <c r="I204" s="9" t="inlineStr"/>
@@ -12422,7 +12422,7 @@
       </c>
       <c r="J213" s="9" t="inlineStr">
         <is>
-          <t>TODO; Scenarios_Method.md</t>
+          <t>TODO; Methods, chapter Macro and results</t>
         </is>
       </c>
       <c r="K213" s="9" t="inlineStr">
@@ -12667,7 +12667,7 @@
       <c r="I218" s="9" t="inlineStr"/>
       <c r="J218" s="9" t="inlineStr">
         <is>
-          <t>check report section 1; PowerModel_Method.md</t>
+          <t>check report section 1; Methods, chapter Power</t>
         </is>
       </c>
       <c r="K218" s="9" t="inlineStr">
@@ -13181,7 +13181,7 @@
       </c>
       <c r="J228" s="9" t="inlineStr">
         <is>
-          <t>GHG_Method.md</t>
+          <t>Methods, chapter Emissions</t>
         </is>
       </c>
       <c r="K228" s="9" t="inlineStr">
@@ -14869,7 +14869,7 @@
       <c r="I260" s="9" t="inlineStr"/>
       <c r="J260" s="9" t="inlineStr">
         <is>
-          <t>Distribution_Method.md</t>
+          <t>Methods, chapter Distribution</t>
         </is>
       </c>
       <c r="K260" s="9" t="inlineStr">
@@ -14914,7 +14914,7 @@
       <c r="I261" s="9" t="inlineStr"/>
       <c r="J261" s="9" t="inlineStr">
         <is>
-          <t>Distribution_Method.md</t>
+          <t>Methods, chapter Distribution</t>
         </is>
       </c>
       <c r="K261" s="9" t="inlineStr">
@@ -14959,7 +14959,7 @@
       <c r="I262" s="9" t="inlineStr"/>
       <c r="J262" s="9" t="inlineStr">
         <is>
-          <t>Distribution_Method.md</t>
+          <t>Methods, chapter Distribution</t>
         </is>
       </c>
       <c r="K262" s="9" t="inlineStr">
@@ -15004,7 +15004,7 @@
       <c r="I263" s="9" t="inlineStr"/>
       <c r="J263" s="9" t="inlineStr">
         <is>
-          <t>Distribution_Method.md</t>
+          <t>Methods, chapter Distribution</t>
         </is>
       </c>
       <c r="K263" s="9" t="inlineStr">
@@ -15049,7 +15049,7 @@
       <c r="I264" s="9" t="inlineStr"/>
       <c r="J264" s="9" t="inlineStr">
         <is>
-          <t>Distribution_Method.md</t>
+          <t>Methods, chapter Distribution</t>
         </is>
       </c>
       <c r="K264" s="9" t="inlineStr">
@@ -15094,7 +15094,7 @@
       <c r="I265" s="9" t="inlineStr"/>
       <c r="J265" s="9" t="inlineStr">
         <is>
-          <t>Distribution_Method.md</t>
+          <t>Methods, chapter Distribution</t>
         </is>
       </c>
       <c r="K265" s="9" t="inlineStr">
@@ -15139,7 +15139,7 @@
       <c r="I266" s="9" t="inlineStr"/>
       <c r="J266" s="9" t="inlineStr">
         <is>
-          <t>Distribution_Method.md</t>
+          <t>Methods, chapter Distribution</t>
         </is>
       </c>
       <c r="K266" s="9" t="inlineStr">
@@ -15184,7 +15184,7 @@
       <c r="I267" s="9" t="inlineStr"/>
       <c r="J267" s="9" t="inlineStr">
         <is>
-          <t>Distribution_Method.md</t>
+          <t>Methods, chapter Distribution</t>
         </is>
       </c>
       <c r="K267" s="9" t="inlineStr">
@@ -15229,7 +15229,7 @@
       <c r="I268" s="9" t="inlineStr"/>
       <c r="J268" s="9" t="inlineStr">
         <is>
-          <t>Distribution_Method.md</t>
+          <t>Methods, chapter Distribution</t>
         </is>
       </c>
       <c r="K268" s="9" t="inlineStr">
@@ -15274,7 +15274,7 @@
       <c r="I269" s="9" t="inlineStr"/>
       <c r="J269" s="9" t="inlineStr">
         <is>
-          <t>Distribution_Method.md</t>
+          <t>Methods, chapter Distribution</t>
         </is>
       </c>
       <c r="K269" s="9" t="inlineStr">

</xml_diff>

<commit_message>
v8.2: register and documents moved to legacy CPAT 1.0pre_465
Row map 456->465 and remap tool; fix plans and register sources remapped and
checked against 465; register v8.2 with the status in legacy of every bug
(CPAT team's fixes: Appendix C confirmed, Appendix B caveats / not fixed);
In legacy 465 columns in BUGS.md, LegacyBugFixes.md and the register
spreadsheet; tracker refreshed. Release v8.2 (workbook formulas unchanged:
quick check 0 change vs v8.1, paste test PASS), deck and Word documentation
rebuilt; tidy-up of bugsfixed/, NORMS, TODO, READMEs, CHANGELOG.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NEaWSMCoGDPkcQwasoKLW3
</commit_message>
<xml_diff>
--- a/excel_ai/CPAT-AI_BugsAndIssues_latest.xlsx
+++ b/excel_ai/CPAT-AI_BugsAndIssues_latest.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUGSandISSUES" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BUGSandISSUES'!$A$3:$K$283</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BUGSandISSUES'!$A$3:$L$283</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -505,7 +505,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUGSandISSUES: CPAT-AI-Mitigation-Prototype v7.0 against legacy CPAT</t>
+          <t>BUGSandISSUES: CPAT-AI-Mitigation-Prototype v8.2 against legacy CPAT</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -538,7 +538,7 @@
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Source: BUGS.md and ISSUES.md (generated from issues_register.py). Not included: potential upgrades (U), and bugs found and fixed in the prototype during development (M); both are in the Word register CPAT-AI_BugsAndIssues_v7.0.docx. Details and effects of the legacy bugs: LegacyBugFixes.md.</t>
+          <t>Source: BUGS.md and ISSUES.md (generated from issues_register.py). Not included: potential upgrades (U), and bugs found and fixed in the prototype during development (M); both are in the Word register CPAT-AI_BugsAndIssues_latest.docx. Details and effects of the legacy bugs: LegacyBugFixes.md. Column "Status in legacy 465": the legacy bugs in the latest CPAT file (CPAT 1.0pre_465), where the CPAT team fixed part of them (checked cell by cell); cell references are 465 rows.</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K283"/>
+  <dimension ref="A1:L283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -801,12 +801,13 @@
     <col width="52" customWidth="1" min="9" max="9"/>
     <col width="38" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bugs and issues of legacy CPAT and whether CPAT-AI-Mitigation-Prototype v7.0 replicates them</t>
+          <t>Bugs and issues of legacy CPAT and whether CPAT-AI-Mitigation-Prototype v8.2 replicates them</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -819,6 +820,7 @@
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -876,6 +878,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>Status in legacy 465</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -933,6 +940,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -990,6 +1002,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -1047,6 +1064,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1104,6 +1126,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1161,6 +1188,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -1218,6 +1250,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -1275,6 +1312,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -1332,6 +1374,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -1389,6 +1436,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -1446,6 +1498,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -1503,6 +1560,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -1560,6 +1622,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -1617,6 +1684,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -1674,6 +1746,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L17" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -1731,6 +1808,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1788,6 +1870,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L19" s="9" t="inlineStr">
+        <is>
+          <t>Fixed with caveats</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -1822,7 +1909,7 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Livestock, rice and waste CH4 are the inventory values divided by the GWP, constant over time; the abatement shares of the methane fee are computed (rows 6182, 6194, 6206) but not applied, so a methane fee on agriculture and waste has no effect.</t>
+          <t>Livestock, rice and waste CH4 are the inventory values divided by the GWP, constant over time; the abatement shares of the methane fee are computed (rows 6168, 6180, 6192) but not applied, so a methane fee on agriculture and waste has no effect.</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
@@ -1832,17 +1919,22 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>Grow livestock, rice and waste methane with their drivers (income, population) and apply the abatement shares already computed in rows 6182, 6194, 6206.</t>
+          <t>Grow livestock, rice and waste methane with their drivers (income, population) and apply the abatement shares already computed in rows 6168, 6180, 6192.</t>
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 6172-6227 (livestock, rice, waste)</t>
+          <t>Mitigation rows 6158-6213 (livestock, rice, waste)</t>
         </is>
       </c>
       <c r="K20" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -1894,12 +1986,17 @@
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 6155-6156</t>
+          <t>Mitigation rows 6141-6142</t>
         </is>
       </c>
       <c r="K21" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -1959,6 +2056,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
@@ -1993,7 +2095,7 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>The abatement share of waste equals that of livestock (=M6182) instead of the waste curve of CH4Inputs.</t>
+          <t>The abatement share of waste equals that of livestock (=M6168) instead of the waste curve of CH4Inputs.</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">
@@ -2003,17 +2105,22 @@
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>Use the waste curve of CH4Inputs for waste (row 6206 now = M6182, the livestock share).</t>
+          <t>Use the waste curve of CH4Inputs for waste (row 6192 now = M6168, the livestock share).</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>Mitigation row 6206</t>
+          <t>Mitigation row 6192</t>
         </is>
       </c>
       <c r="K23" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2073,6 +2180,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L24" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
@@ -2122,12 +2234,17 @@
       </c>
       <c r="J25" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 6704, 6806, ... (total emissions of each pollutant)</t>
+          <t>Mitigation rows 6690, 6792, ... (total emissions of each pollutant)</t>
         </is>
       </c>
       <c r="K25" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L25" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2179,12 +2296,17 @@
       </c>
       <c r="J26" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 2443-2446, 8288</t>
+          <t>Mitigation rows 2443-2446, 8274</t>
         </is>
       </c>
       <c r="K26" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2244,6 +2366,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L27" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -2301,6 +2428,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L28" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -2358,6 +2490,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L29" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
@@ -2415,6 +2552,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L30" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
@@ -2472,6 +2614,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L31" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
@@ -2529,6 +2676,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L32" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
@@ -2586,6 +2738,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L33" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
@@ -2643,6 +2800,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L34" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
@@ -2700,6 +2862,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L35" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
@@ -2757,6 +2924,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L36" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
@@ -2814,6 +2986,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L37" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
@@ -2871,6 +3048,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L38" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
@@ -2928,6 +3110,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L39" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
@@ -2985,6 +3172,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L40" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -3042,6 +3234,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L41" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
@@ -3099,6 +3296,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L42" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
@@ -3156,6 +3358,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L43" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
@@ -3213,6 +3420,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L44" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
@@ -3247,7 +3459,7 @@
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>The income factor points to the blank row 2440, so other energy use never grows with GDP; rows 6077-6084 have no additional-efficiency term.</t>
+          <t>The income factor points to the blank row 2440, so other energy use never grows with GDP; rows 6063-6070 have no additional-efficiency term.</t>
         </is>
       </c>
       <c r="H45" s="9" t="inlineStr">
@@ -3262,12 +3474,17 @@
       </c>
       <c r="J45" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 6077-6085</t>
+          <t>Mitigation rows 6063-6071</t>
         </is>
       </c>
       <c r="K45" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L45" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3327,6 +3544,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L46" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
@@ -3384,6 +3606,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L47" s="9" t="inlineStr">
+        <is>
+          <t>Fixed with caveats</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
@@ -3441,6 +3668,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L48" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
@@ -3498,6 +3730,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L49" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
@@ -3555,6 +3792,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L50" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
@@ -3604,12 +3846,17 @@
       </c>
       <c r="J51" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 18177-18181, 742</t>
+          <t>Mitigation rows 18162-18166, 742</t>
         </is>
       </c>
       <c r="K51" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L51" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3661,12 +3908,17 @@
       </c>
       <c r="J52" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 18195-18213</t>
+          <t>Mitigation rows 18180-18198</t>
         </is>
       </c>
       <c r="K52" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L52" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3726,6 +3978,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L53" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
@@ -3783,6 +4040,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L54" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
@@ -3840,6 +4102,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L55" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
@@ -3897,6 +4164,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L56" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
@@ -3954,6 +4226,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L57" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
@@ -4011,6 +4288,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L58" s="9" t="inlineStr">
+        <is>
+          <t>Fixed with caveats</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
@@ -4068,6 +4350,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L59" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
@@ -4117,12 +4404,17 @@
       </c>
       <c r="J60" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 15900-16700 (GAINS factor lookups)</t>
+          <t>Mitigation rows 15885-16685 (GAINS factor lookups)</t>
         </is>
       </c>
       <c r="K60" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L60" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4451,7 @@
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>A fuel that its GAINS subsector has no factor for gets 0, although it burns: Egypt 2022 residential LPG (3,182 ktoe), other mining diesel (3,819), food &amp; forestry diesel (927), fuel transformation LPG (2,466); food &amp; forestry shows about 1 t of NOx (legacy row 15939).</t>
+          <t>A fuel that its GAINS subsector has no factor for gets 0, although it burns: Egypt 2022 residential LPG (3,182 ktoe), other mining diesel (3,819), food &amp; forestry diesel (927), fuel transformation LPG (2,466); food &amp; forestry shows about 1 t of NOx (legacy row 15924).</t>
         </is>
       </c>
       <c r="H61" s="9" t="inlineStr">
@@ -4174,12 +4466,17 @@
       </c>
       <c r="J61" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 15900-16700 (GAINS factor lookups; sheet EF_PM)</t>
+          <t>Mitigation rows 15885-16685 (GAINS factor lookups; sheet EF_PM)</t>
         </is>
       </c>
       <c r="K61" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L61" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4239,6 +4536,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L62" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
@@ -4296,6 +4598,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L63" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
@@ -4353,6 +4660,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L64" s="9" t="inlineStr">
+        <is>
+          <t>Not fixed (marked fixed)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
@@ -4410,6 +4722,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L65" s="9" t="inlineStr">
+        <is>
+          <t>Not fixed (marked fixed)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
@@ -4467,6 +4784,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L66" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
@@ -4524,6 +4846,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L67" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
@@ -4581,6 +4908,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L68" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="9" t="inlineStr">
@@ -4638,6 +4970,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L69" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="9" t="inlineStr">
@@ -4687,12 +5024,17 @@
       </c>
       <c r="J70" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 8267-8288 (policy 14584-14605)</t>
+          <t>Mitigation rows 8253-8274 (policy 14569-14590)</t>
         </is>
       </c>
       <c r="K70" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L70" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4729,7 +5071,7 @@
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>The excise (revenue) use of the first cohort looks up L$8127, a baseline-block cell (0), instead of the cohort's own row (L14387); the contractionary effect of the first year's revenue is dropped (Egypt about 3e-5 of GDP).</t>
+          <t>The excise (revenue) use of the first cohort looks up L$8113, a baseline-block cell (0), instead of the cohort's own row (L14372); the contractionary effect of the first year's revenue is dropped (Egypt about 3e-5 of GDP).</t>
         </is>
       </c>
       <c r="H71" s="9" t="inlineStr">
@@ -4739,17 +5081,22 @@
       </c>
       <c r="I71" s="9" t="inlineStr">
         <is>
-          <t>Match the first cohort's excise use on its own row (L14387, baseline L8070), not L$8127.</t>
+          <t>Match the first cohort's excise use on its own row (L14372, baseline L8056), not L$8113.</t>
         </is>
       </c>
       <c r="J71" s="9" t="inlineStr">
         <is>
-          <t>Mitigation row 8071 (policy 14388)</t>
+          <t>Mitigation row 8057 (policy 14373)</t>
         </is>
       </c>
       <c r="K71" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L71" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4786,7 +5133,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>The additional excise of gas in industry is the coal industry tax (R2512) x coal industry use (R6436).</t>
+          <t>The additional excise of gas in industry is the coal industry tax (R2512) x coal industry use (R6422).</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4796,17 +5143,22 @@
       </c>
       <c r="I72" s="9" t="inlineStr">
         <is>
-          <t>Use the gas industry excise rate (row 2581) and gas industry use in row 7761.</t>
+          <t>Use the gas industry excise rate (row 2581) and gas industry use in row 7747.</t>
         </is>
       </c>
       <c r="J72" s="9" t="inlineStr">
         <is>
-          <t>Mitigation row 7761 (policy 14078)</t>
+          <t>Mitigation row 7747 (policy 14063)</t>
         </is>
       </c>
       <c r="K72" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L72" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4853,17 +5205,22 @@
       </c>
       <c r="I73" s="9" t="inlineStr">
         <is>
-          <t>Multiply by _conv_ktoe_to_gj in rows 7805, 7819, 7873.</t>
+          <t>Multiply by _conv_ktoe_to_gj in rows 7791, 7805, 7859.</t>
         </is>
       </c>
       <c r="J73" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 7805, 7819, 7873</t>
+          <t>Mitigation rows 7791, 7805, 7859</t>
         </is>
       </c>
       <c r="K73" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L73" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4910,17 +5267,22 @@
       </c>
       <c r="I74" s="9" t="inlineStr">
         <is>
-          <t>Read column R (the year) in rows 7671 and 7756.</t>
+          <t>Read column R (the year) in rows 7657 and 7742.</t>
         </is>
       </c>
       <c r="J74" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 7671, 7756</t>
+          <t>Mitigation rows 7657, 7742</t>
         </is>
       </c>
       <c r="K74" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L74" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4957,7 +5319,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>Gas industry coverage divides by R6041 instead of the industry gas total (6442); kerosene power coverage multiplies power by domestic shipping (R2270 x R2273).</t>
+          <t>Gas industry coverage divides by R6027 instead of the industry gas total (6428); kerosene power coverage multiplies power by domestic shipping (R2270 x R2273).</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -4967,17 +5329,22 @@
       </c>
       <c r="I75" s="9" t="inlineStr">
         <is>
-          <t>Divide by the industry gas total (6442) in row 7691; use power x kerosene coverage (R2265 x R2270) in row 7718.</t>
+          <t>Divide by the industry gas total (6428) in row 7677; use power x kerosene coverage (R2265 x R2270) in row 7704.</t>
         </is>
       </c>
       <c r="J75" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 7691 (policy 14008), 7718</t>
+          <t>Mitigation rows 7677 (policy 13993), 7704</t>
         </is>
       </c>
       <c r="K75" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L75" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5029,12 +5396,17 @@
       </c>
       <c r="J76" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 17160-17164, 17190, 17201</t>
+          <t>Mitigation rows 17145-17149, 17175, 17186</t>
         </is>
       </c>
       <c r="K76" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L76" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5094,6 +5466,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L77" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="9" t="inlineStr">
@@ -5128,7 +5505,7 @@
       </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>The "indexed vs 2022" rows read rows 16331-16338 (electricity industry, electricity residential, coal industry, ...) under the labels electricity, coal, gas, oil, ...; E16317 tests the policy gas total instead of the baseline one; labels say 2022 = 100 where baseline = 100.</t>
+          <t>The "indexed vs 2022" rows read rows 16316-16323 (electricity industry, electricity residential, coal industry, ...) under the labels electricity, coal, gas, oil, ...; E16302 tests the policy gas total instead of the baseline one; labels say 2022 = 100 where baseline = 100.</t>
         </is>
       </c>
       <c r="H78" s="9" t="inlineStr">
@@ -5138,17 +5515,22 @@
       </c>
       <c r="I78" s="9" t="inlineStr">
         <is>
-          <t>Point rows 16398-16405 to the average-price rows of each fuel; test the baseline gas total in E16317; relabel "baseline = 100".</t>
+          <t>Point rows 16383-16390 to the average-price rows of each fuel; test the baseline gas total in E16302; relabel "baseline = 100".</t>
         </is>
       </c>
       <c r="J78" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 16317, 16389-16405</t>
+          <t>Mitigation rows 16302, 16374-16390</t>
         </is>
       </c>
       <c r="K78" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L78" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5208,6 +5590,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L79" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="9" t="inlineStr">
@@ -5257,12 +5644,17 @@
       </c>
       <c r="J80" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 2322-2325 (policy 8653-8656), 7789-7792</t>
+          <t>Mitigation rows 2322-2325 (policy 8638-8641), 7775-7778</t>
         </is>
       </c>
       <c r="K80" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L80" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5322,6 +5714,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L81" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="9" t="inlineStr">
@@ -5379,6 +5776,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L82" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="9" t="inlineStr">
@@ -5436,6 +5838,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L83" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="9" t="inlineStr">
@@ -5493,6 +5900,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L84" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="9" t="inlineStr">
@@ -5550,6 +5962,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L85" s="9" t="inlineStr">
+        <is>
+          <t>Fixed with caveats</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="9" t="inlineStr">
@@ -5599,12 +6016,17 @@
       </c>
       <c r="J86" s="9" t="inlineStr">
         <is>
-          <t>Mitigation row 7820</t>
+          <t>Mitigation row 7806</t>
         </is>
       </c>
       <c r="K86" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L86" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5664,6 +6086,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L87" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="9" t="inlineStr">
@@ -5721,6 +6148,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L88" s="9" t="inlineStr">
+        <is>
+          <t>Fixed with caveats</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="9" t="inlineStr">
@@ -5778,6 +6210,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L89" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="9" t="inlineStr">
@@ -5835,6 +6272,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L90" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="9" t="inlineStr">
@@ -5892,6 +6334,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L91" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="9" t="inlineStr">
@@ -5949,6 +6396,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L92" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="9" t="inlineStr">
@@ -6006,6 +6458,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L93" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="9" t="inlineStr">
@@ -6063,6 +6520,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L94" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="9" t="inlineStr">
@@ -6120,6 +6582,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L95" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="9" t="inlineStr">
@@ -6177,6 +6644,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L96" s="9" t="inlineStr">
+        <is>
+          <t>Fixed with caveats</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="9" t="inlineStr">
@@ -6226,12 +6698,17 @@
       </c>
       <c r="J97" s="9" t="inlineStr">
         <is>
-          <t>Mitigation C2199:C2201 ('Tax in nominal or real terms?', 'Exponential option or linear' twice) beside K2199:M2201 (road, residential, industrial additional efficiency, MTInputs F243-F245); E2385 (LPG 'Road'), E2386 (kerosene 'Industry') on all-sector rows (codes shp.lpg.all, shp.ker.all); D5615, D5722, D6072, D6083 'Other oil pinducts'</t>
+          <t>Mitigation C2199:C2201 ('Tax in nominal or real terms?', 'Exponential option or linear' twice) beside K2199:M2201 (road, residential, industrial additional efficiency, MTInputs F243-F245); E2385 (LPG 'Road'), E2386 (kerosene 'Industry') on all-sector rows (codes shp.lpg.all, shp.ker.all); D5615, D5711, D6058, D6069 'Other oil pinducts'</t>
         </is>
       </c>
       <c r="K97" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L97" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6268,7 +6745,7 @@
       </c>
       <c r="G98" s="9" t="inlineStr">
         <is>
-          <t>An EF-weighted average price (5714), an elasticity table (5668-5676) and 'Fuel'/'Average' demand and efficiency multiples (5727-5728) are computed but referenced nowhere; M5667 takes next year's GDP growth (N2446).</t>
+          <t>An EF-weighted average price (5703), an elasticity table (5668-5676) and 'Fuel'/'Average' demand and efficiency multiples (5727-5728) are computed but referenced nowhere; M5667 takes next year's GDP growth (N2446).</t>
         </is>
       </c>
       <c r="H98" s="9" t="inlineStr">
@@ -6283,12 +6760,17 @@
       </c>
       <c r="J98" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 5667-5676, 5714, 5727-5728 (iron &amp; steel block; M5667 = N2446)</t>
+          <t>Mitigation rows 5667-5676, 5703, 5727-5728 (iron &amp; steel block; M5667 = N2446)</t>
         </is>
       </c>
       <c r="K98" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L98" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6348,6 +6830,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L99" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="9" t="inlineStr">
@@ -6405,6 +6892,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L100" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="9" t="inlineStr">
@@ -6462,6 +6954,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L101" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="9" t="inlineStr">
@@ -6519,6 +7016,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L102" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="9" t="inlineStr">
@@ -6576,6 +7078,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L103" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="9" t="inlineStr">
@@ -6610,7 +7117,7 @@
       </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
-          <t>The SCC block of Manual inputs is read by nothing; the Manual option of NSCCSource / GSCCSource takes the path typed on Mitigation row 17683.</t>
+          <t>The SCC block of Manual inputs is read by nothing; the Manual option of NSCCSource / GSCCSource takes the path typed on Mitigation row 17668.</t>
         </is>
       </c>
       <c r="H104" s="9" t="inlineStr">
@@ -6620,17 +7127,22 @@
       </c>
       <c r="I104" s="9" t="inlineStr">
         <is>
-          <t>Mitigation row 17683 = 'Manual inputs'!J237 (NSCC) / J240 (GSCC).</t>
+          <t>Mitigation row 17668 = 'Manual inputs'!J237 (NSCC) / J240 (GSCC).</t>
         </is>
       </c>
       <c r="J104" s="9" t="inlineStr">
         <is>
-          <t>Manual inputs rows 234-240; Mitigation row 17683</t>
+          <t>Manual inputs rows 234-240; Mitigation row 17668</t>
         </is>
       </c>
       <c r="K104" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L104" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6690,6 +7202,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L105" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="9" t="inlineStr">
@@ -6747,6 +7264,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L106" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="9" t="inlineStr">
@@ -6804,6 +7326,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L107" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="9" t="inlineStr">
@@ -6838,7 +7365,7 @@
       </c>
       <c r="G108" s="9" t="inlineStr">
         <is>
-          <t>The additional renewable subsidy (MTInputs 355) starts in the year the consumer fuel subsidies start to be phased out; it has no start-year input of its own.</t>
+          <t>The additional renewable subsidy (MTInputs 353) starts in the year the consumer fuel subsidies start to be phased out; it has no start-year input of its own.</t>
         </is>
       </c>
       <c r="H108" s="9" t="inlineStr">
@@ -6853,12 +7380,17 @@
       </c>
       <c r="J108" s="9" t="inlineStr">
         <is>
-          <t>Mitigation E2736 (policy E9067) = row 270 = MTInputs F132 (YearConsSubPha)</t>
+          <t>Mitigation E2736 (policy E9052) = row 270 = MTInputs F132 (YearConsSubPha)</t>
         </is>
       </c>
       <c r="K108" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L108" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6895,7 +7427,7 @@
       </c>
       <c r="G109" s="9" t="inlineStr">
         <is>
-          <t>Rows 7897-7900 = (row 2743 + row 2745) x generation, but row 2745 already equals row 2743 minus the additional subsidy, so the base subsidy enters twice; hydro (7899) ignores RenewableSubsidyHydro; biomass has no row; 7903 enters total revenue (row 8023).</t>
+          <t>Rows 7883-7886 = (row 2743 + row 2745) x generation, but row 2745 already equals row 2743 minus the additional subsidy, so the base subsidy enters twice; hydro (7885) ignores RenewableSubsidyHydro; biomass has no row; 7889 enters total revenue (row 8009).</t>
         </is>
       </c>
       <c r="H109" s="9" t="inlineStr">
@@ -6905,17 +7437,22 @@
       </c>
       <c r="I109" s="9" t="inlineStr">
         <is>
-          <t>Rows 7897-7901 = the subsidy by type (rows 3148-3152) x generation.</t>
+          <t>Rows 7883-7887 = the subsidy by type (rows 3148-3152) x generation.</t>
         </is>
       </c>
       <c r="J109" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 7897-7903 (policy +6317)</t>
+          <t>Mitigation rows 7883-7889 (policy +6316)</t>
         </is>
       </c>
       <c r="K109" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L109" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6975,6 +7512,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L110" s="9" t="inlineStr">
+        <is>
+          <t>Fixed with caveats</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="9" t="inlineStr">
@@ -7009,7 +7551,7 @@
       </c>
       <c r="G111" s="9" t="inlineStr">
         <is>
-          <t>The rebate includes VAT (carbon cost x pass-through x (1 + VAT)) and enters total revenue through row 7749, while the VAT on the carbon cost is never counted as revenue.</t>
+          <t>The rebate includes VAT (carbon cost x pass-through x (1 + VAT)) and enters total revenue through row 7735, while the VAT on the carbon cost is never counted as revenue.</t>
         </is>
       </c>
       <c r="H111" s="9" t="inlineStr">
@@ -7024,12 +7566,17 @@
       </c>
       <c r="J111" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 3615, 3644, 3663, 7888, 7749 (policy +6331 / +6317)</t>
+          <t>Mitigation rows 3615, 3644, 3663, 7874, 7735 (policy +6316 / +6316)</t>
         </is>
       </c>
       <c r="K111" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L111" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -7066,7 +7613,7 @@
       </c>
       <c r="G112" s="9" t="inlineStr">
         <is>
-          <t>The revenue memo 3660 (and 7762) = manual excise x consumption in every year, while the price includes only the change since the last historical year x pass-through.</t>
+          <t>The revenue memo 3660 (and 7748) = manual excise x consumption in every year, while the price includes only the change since the last historical year x pass-through.</t>
         </is>
       </c>
       <c r="H112" s="9" t="inlineStr">
@@ -7081,12 +7628,17 @@
       </c>
       <c r="J112" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 3602, 3631, 3660, 7885, 7762</t>
+          <t>Mitigation rows 3602, 3631, 3660, 7871, 7748</t>
         </is>
       </c>
       <c r="K112" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L112" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -7133,17 +7685,22 @@
       </c>
       <c r="I113" s="9" t="inlineStr">
         <is>
-          <t>In rows 8708-8719 refer to the policy block ($D$8700, L$8706) instead of $D$2369 and L$2375.</t>
+          <t>In rows 8693-8704 refer to the policy block ($D$8685, L$8691) instead of $D$2369 and L$2375.</t>
         </is>
       </c>
       <c r="J113" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 8708-8719 (policy copies of 2377-2388)</t>
+          <t>Mitigation rows 8693-8704 (policy copies of 2377-2388)</t>
         </is>
       </c>
       <c r="K113" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L113" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -7203,6 +7760,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L114" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
@@ -7237,7 +7799,7 @@
       </c>
       <c r="G115" s="9" t="inlineStr">
         <is>
-          <t>MTInputs 354-355 are labelled $/kWh nominal but enter the real cost and revenue without deflation (row 2743 = -E2734). A formula that contradicts its label: reclassified as a bug by the user (2026-10-19).</t>
+          <t>MTInputs 352-353 are labelled $/kWh nominal but enter the real cost and revenue without deflation (row 2743 = -E2734). A formula that contradicts its label: reclassified as a bug by the user (2026-10-19).</t>
         </is>
       </c>
       <c r="H115" s="9" t="inlineStr">
@@ -7247,17 +7809,22 @@
       </c>
       <c r="I115" s="9" t="inlineStr">
         <is>
-          <t>Deflate the nominal inputs (rows 2734-2735) by the CPI index before they enter row 2743, or relabel MTInputs 354-355 as real.</t>
+          <t>Deflate the nominal inputs (rows 2734-2735) by the CPI index before they enter row 2743, or relabel MTInputs 352-353 as real.</t>
         </is>
       </c>
       <c r="J115" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 2734-2735, 2743, 2745 (MTInputs 354-355)</t>
+          <t>Mitigation rows 2734-2735, 2743, 2745 (MTInputs 352-353)</t>
         </is>
       </c>
       <c r="K115" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L115" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -7304,17 +7871,22 @@
       </c>
       <c r="I116" s="9" t="inlineStr">
         <is>
-          <t>Point row 2555 (and policy 8886) at the residential gas ETS row 1715.</t>
+          <t>Point row 2555 (and policy 8871) at the residential gas ETS row 1715.</t>
         </is>
       </c>
       <c r="J116" s="9" t="inlineStr">
         <is>
-          <t>Mitigation row 2555 (policy 8886)</t>
+          <t>Mitigation row 2555 (policy 8871)</t>
         </is>
       </c>
       <c r="K116" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L116" s="9" t="inlineStr">
+        <is>
+          <t>Fixed with caveats</t>
         </is>
       </c>
     </row>
@@ -7374,6 +7946,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L117" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="9" t="inlineStr">
@@ -7431,6 +8008,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L118" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="9" t="inlineStr">
@@ -7488,6 +8070,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L119" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="9" t="inlineStr">
@@ -7522,7 +8109,7 @@
       </c>
       <c r="G120" s="9" t="inlineStr">
         <is>
-          <t>F18414 = IF(target year &lt; 2030, (2030 - base)/(target year - base), 1) is at least 1, so the "&lt;1" branches of the Fixed and Historical blocks (rows 18441-18443, 18458-18460) never run, while the BAU block multiplies both the reduction (18422) and the level (18425: BAU x (1 - reduction x adj) x adj) by it: a 2025 BAU target is scaled up twice and the other types not at all. Found by the item 8 plan (v5.7).</t>
+          <t>F18399 = IF(target year &lt; 2030, (2030 - base)/(target year - base), 1) is at least 1, so the "&lt;1" branches of the Fixed and Historical blocks (rows 18426-18428, 18443-18445) never run, while the BAU block multiplies both the reduction (18407) and the level (18410: BAU x (1 - reduction x adj) x adj) by it: a 2025 BAU target is scaled up twice and the other types not at all. Found by the item 8 plan (v5.7).</t>
         </is>
       </c>
       <c r="H120" s="9" t="inlineStr">
@@ -7537,12 +8124,17 @@
       </c>
       <c r="J120" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 18414, 18422-18427, 18441-18443, 18458-18460</t>
+          <t>Mitigation rows 18399, 18407-18412, 18426-18428, 18443-18445</t>
         </is>
       </c>
       <c r="K120" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L120" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -7579,7 +8171,7 @@
       </c>
       <c r="G121" s="9" t="inlineStr">
         <is>
-          <t>Rows 18497-18498 divide the start-year emissions by the target (G18446/F18494) while row 18499 divides the target by the start-year emissions; the chart rows 18509-18510 read 18499 for the unconditional line and 18498 (inverted) for the conditional one. Found by the item 8 plan (v5.7).</t>
+          <t>Rows 18482-18483 divide the start-year emissions by the target (G18431/F18479) while row 18484 divides the target by the start-year emissions; the chart rows 18494-18495 read 18484 for the unconditional line and 18483 (inverted) for the conditional one. Found by the item 8 plan (v5.7).</t>
         </is>
       </c>
       <c r="H121" s="9" t="inlineStr">
@@ -7589,17 +8181,22 @@
       </c>
       <c r="I121" s="9" t="inlineStr">
         <is>
-          <t>Use target / start-year emissions in rows 18497-18498, as 18499.</t>
+          <t>Use target / start-year emissions in rows 18482-18483, as 18484.</t>
         </is>
       </c>
       <c r="J121" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 18497-18499</t>
+          <t>Mitigation rows 18482-18484</t>
         </is>
       </c>
       <c r="K121" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L121" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -7636,7 +8233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>Rows 18458-18460 return the cut (F18455 x adj) when adj &lt; 1 and the level otherwise; harmless today only because adj &lt; 1 never happens (L119). Found by the item 8 plan (v5.7).</t>
+          <t>Rows 18443-18445 return the cut (F18440 x adj) when adj &lt; 1 and the level otherwise; harmless today only because adj &lt; 1 never happens (L119). Found by the item 8 plan (v5.7).</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -7646,17 +8243,22 @@
       </c>
       <c r="I122" s="9" t="inlineStr">
         <is>
-          <t>Return F18452 - F18455 x adj (the level), as the Fixed block.</t>
+          <t>Return F18437 - F18440 x adj (the level), as the Fixed block.</t>
         </is>
       </c>
       <c r="J122" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 18458-18460</t>
+          <t>Mitigation rows 18443-18445</t>
         </is>
       </c>
       <c r="K122" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L122" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -7693,7 +8295,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>The excludes-LULUCF branch adds $J$18465 where the LULUCF emissions are in column I (I18465 = G - F). J18465 is not blank: it holds the non-CO2 emissions (F - H, 254.9 Mt for Egypt), so non-CO2 is counted twice and LULUCF is missed (cell plan 2026-10-20 corrected the register). Found by the item 8 plan (v5.7).</t>
+          <t>The excludes-LULUCF branch adds $J$18450 where the LULUCF emissions are in column I (I18450 = G - F). J18450 is not blank: it holds the non-CO2 emissions (F - H, 254.9 Mt for Egypt), so non-CO2 is counted twice and LULUCF is missed (cell plan 2026-10-20 corrected the register). Found by the item 8 plan (v5.7).</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -7703,17 +8305,22 @@
       </c>
       <c r="I123" s="9" t="inlineStr">
         <is>
-          <t>Add I18465 (LULUCF) instead of J18465 (non-CO2).</t>
+          <t>Add I18450 (LULUCF) instead of J18450 (non-CO2).</t>
         </is>
       </c>
       <c r="J123" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 18476-18477</t>
+          <t>Mitigation rows 18461-18462</t>
         </is>
       </c>
       <c r="K123" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L123" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -7765,12 +8372,17 @@
       </c>
       <c r="J124" s="9" t="inlineStr">
         <is>
-          <t>Mitigation row 18466</t>
+          <t>Mitigation row 18451</t>
         </is>
       </c>
       <c r="K124" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L124" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -7830,6 +8442,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L125" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="9" t="inlineStr">
@@ -7887,6 +8504,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L126" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="9" t="inlineStr">
@@ -7944,6 +8566,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L127" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="9" t="inlineStr">
@@ -8001,6 +8628,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L128" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="9" t="inlineStr">
@@ -8035,27 +8667,32 @@
       </c>
       <c r="G129" s="9" t="inlineStr">
         <is>
-          <t>The net revenue rows (USD and % of GDP) read the next column of rows 8038 and 8043 (K6252 = L8038 ... AD6252 = AE8038), so each year shows the next year's net revenue. Report only (rows 6253, 6258 read them). Found by the read-of-later-years scan of legacy (v6.2, user 2026-10-20).</t>
+          <t>The net revenue rows (USD and % of GDP) read the next column of rows 8024 and 8029 (K6238 = L8024 ... AD6238 = AE8024), so each year shows the next year's net revenue. Report only (rows 6239, 6244 read them). Found by the read-of-later-years scan of legacy (v6.2, user 2026-10-20).</t>
         </is>
       </c>
       <c r="H129" s="9" t="inlineStr">
         <is>
-          <t>Each year reports the next year's net revenue (USD and % of GDP). prototype: Not in the prototype (its revenue rows read the same year; reporting rebuilt). Legacy fix: K6252 =K8038 and K6257 =K8043, filled K:AD.</t>
+          <t>Each year reports the next year's net revenue (USD and % of GDP). prototype: Not in the prototype (its revenue rows read the same year; reporting rebuilt). Legacy fix: K6238 =K8024 and K6243 =K8029, filled K:AD.</t>
         </is>
       </c>
       <c r="I129" s="9" t="inlineStr">
         <is>
-          <t>K6252 =K8038 and K6257 =K8043, filled K:AD; policy rows 12569, 12574 the same (+6,317).</t>
+          <t>K6238 =K8024 and K6243 =K8029, filled K:AD; policy rows 12554, 12559 the same (+6,316).</t>
         </is>
       </c>
       <c r="J129" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 6252, 6257 (policy 12569, 12574)</t>
+          <t>Mitigation rows 6238, 6243 (policy 12554, 12559)</t>
         </is>
       </c>
       <c r="K129" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L129" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -8092,27 +8729,32 @@
       </c>
       <c r="G130" s="9" t="inlineStr">
         <is>
-          <t>The rows add L2743 + L2745, but L2745 already includes L2743, so the baseline renewable subsidy is counted twice. Only when MTInputs row 354 (RenewableSubsidyBL) is not zero; 0 for Egypt. Found by the cell plans (user 2026-10-20: a bug).</t>
+          <t>The rows add L2743 + L2745, but L2745 already includes L2743, so the baseline renewable subsidy is counted twice. Only when MTInputs row 352 (RenewableSubsidyBL) is not zero; 0 for Egypt. Found by the cell plans (user 2026-10-20: a bug).</t>
         </is>
       </c>
       <c r="H130" s="9" t="inlineStr">
         <is>
-          <t>With a baseline renewable subsidy (MTInputs 354) the subsidy cost is counted twice. prototype: Fixed (prototype: one renewable subsidy row rnsp = baseline + additional, counted once).</t>
+          <t>With a baseline renewable subsidy (MTInputs 352) the subsidy cost is counted twice. prototype: Fixed (prototype: one renewable subsidy row rnsp = baseline + additional, counted once).</t>
         </is>
       </c>
       <c r="I130" s="9" t="inlineStr">
         <is>
-          <t>In rows 2785-2788, 2947-2951 and 7897-7900 drop the + L2743 term (L2745 already includes it); policy rows the same (+6,331).</t>
+          <t>In rows 2785-2788, 2947-2951 and 7883-7886 drop the + L2743 term (L2745 already includes it); policy rows the same (+6,316).</t>
         </is>
       </c>
       <c r="J130" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 2785-2788, 2947-2951, 7897-7900 (against 2743, 2745)</t>
+          <t>Mitigation rows 2785-2788, 2947-2951, 7883-7886 (against 2743, 2745)</t>
         </is>
       </c>
       <c r="K130" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L130" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8149,7 +8791,7 @@
       </c>
       <c r="G131" s="9" t="inlineStr">
         <is>
-          <t>F18471 (conditional) applies the cut to the target-year BAU intensity (F18469); F18470 (unconditional) applies it to the reference-year intensity (F18468). Found by the cell plans (user 2026-10-20: a bug).</t>
+          <t>F18456 (conditional) applies the cut to the target-year BAU intensity (F18454); F18455 (unconditional) applies it to the reference-year intensity (F18453). Found by the cell plans (user 2026-10-20: a bug).</t>
         </is>
       </c>
       <c r="H131" s="9" t="inlineStr">
@@ -8159,17 +8801,22 @@
       </c>
       <c r="I131" s="9" t="inlineStr">
         <is>
-          <t>F18471: apply the cut to the reference-year intensity F18468, as F18470 does.</t>
+          <t>F18456: apply the cut to the reference-year intensity F18453, as F18455 does.</t>
         </is>
       </c>
       <c r="J131" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 18470-18471</t>
+          <t>Mitigation rows 18455-18456</t>
         </is>
       </c>
       <c r="K131" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L131" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8221,12 +8868,17 @@
       </c>
       <c r="J132" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 466, 2442, 16185 (gdp.pre.lvl); 7736, 7756, 7999 (sub.new.usd); 7652-13977 (rev.ctr.coa)</t>
+          <t>Mitigation rows 466, 2442, 16170 (gdp.pre.lvl); 7722, 7742, 7985 (sub.new.usd); 7638-13962 (rev.ctr.coa)</t>
         </is>
       </c>
       <c r="K132" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L132" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8278,12 +8930,17 @@
       </c>
       <c r="J133" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 7620, 13937 (oc.tot.); em.pm2.All.&lt;sector&gt; rows</t>
+          <t>Mitigation rows 7606, 13922 (oc.tot.); em.pm2.All.&lt;sector&gt; rows</t>
         </is>
       </c>
       <c r="K133" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L133" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8335,12 +8992,17 @@
       </c>
       <c r="J134" s="9" t="inlineStr">
         <is>
-          <t>Mitigation rows 7620, 13937 and the GHG total rows (nox.tot)</t>
+          <t>Mitigation rows 7606, 13922 and the GHG total rows (nox.tot)</t>
         </is>
       </c>
       <c r="K134" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L134" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8396,6 +9058,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L135" s="9" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="9" t="inlineStr">
@@ -8449,6 +9112,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L136" s="9" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="9" t="inlineStr">
@@ -8502,6 +9166,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L137" s="9" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="9" t="inlineStr">
@@ -8536,7 +9201,7 @@
       </c>
       <c r="G138" s="9" t="inlineStr">
         <is>
-          <t>Legacy counts the methane fee in total revenue (row 8024) and so in the fiscal space, on the scenario's own activity. The prototype counts it too, but with the stored scenario-1 activity of downstream gas and biomass use (v6.2, user decision 2026-10-20: no vulnerability to circular references through the GDP feedback). Differs from legacy only when a policy changes gas or biomass use and a methane fee applies. None for Egypt (no methane fee in the scenarios).</t>
+          <t>Legacy counts the methane fee in total revenue (row 8010) and so in the fiscal space, on the scenario's own activity. The prototype counts it too, but with the stored scenario-1 activity of downstream gas and biomass use (v6.2, user decision 2026-10-20: no vulnerability to circular references through the GDP feedback). Differs from legacy only when a policy changes gas or biomass use and a methane fee applies. None for Egypt (no methane fee in the scenarios).</t>
         </is>
       </c>
       <c r="H138" s="9" t="inlineStr"/>
@@ -8555,6 +9220,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L138" s="9" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="9" t="inlineStr">
@@ -8608,6 +9274,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L139" s="9" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="9" t="inlineStr">
@@ -8661,6 +9328,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L140" s="9" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="9" t="inlineStr">
@@ -8714,6 +9382,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L141" s="9" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="9" t="inlineStr">
@@ -8767,6 +9436,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L142" s="9" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="9" t="inlineStr">
@@ -8820,6 +9490,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L143" s="9" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="9" t="inlineStr">
@@ -8854,7 +9525,7 @@
       </c>
       <c r="G144" s="9" t="inlineStr">
         <is>
-          <t>Legacy row 18464 H uses 5665 (Mt CO2) for China instead of the data (row 889). The prototype reads sheet GHGHist (or the model where the reference year is modelled); China's latest NDC is a Historical target (ref 2024, modelled), so the value is not used.</t>
+          <t>Legacy row 18449 H uses 5665 (Mt CO2) for China instead of the data (row 889). The prototype reads sheet GHGHist (or the model where the reference year is modelled); China's latest NDC is a Historical target (ref 2024, modelled), so the value is not used.</t>
         </is>
       </c>
       <c r="H144" s="9" t="inlineStr"/>
@@ -8873,6 +9544,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L144" s="9" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="9" t="inlineStr">
@@ -8926,6 +9598,7 @@
           <t>Dropped</t>
         </is>
       </c>
+      <c r="L145" s="9" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="9" t="inlineStr">
@@ -8979,6 +9652,7 @@
           <t>Dropped</t>
         </is>
       </c>
+      <c r="L146" s="9" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
@@ -9032,6 +9706,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L147" s="9" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="9" t="inlineStr">
@@ -9085,6 +9760,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L148" s="9" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="9" t="inlineStr">
@@ -9138,6 +9814,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L149" s="9" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="9" t="inlineStr">
@@ -9191,6 +9868,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L150" s="9" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="9" t="inlineStr">
@@ -9244,6 +9922,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L151" s="9" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="9" t="inlineStr">
@@ -9297,6 +9976,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L152" s="9" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="9" t="inlineStr">
@@ -9350,6 +10030,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L153" s="9" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="9" t="inlineStr">
@@ -9390,7 +10071,7 @@
       <c r="H154" s="9" t="inlineStr"/>
       <c r="I154" s="9" t="inlineStr">
         <is>
-          <t>Traced (v5.6): legacy process emissions = 2023 inventory x the year-on-year growth of industrial energy CO2 (row 6590; 2024: +16.8%, the rebound after the 2023 demand shock, so 56.9 -&gt; 66.5). The prototype floored that growth at 0 (a departure: removed in v5.6, as legacy). The remaining gap is the industrial energy CO2 path, part of the fuel-use gap (I14).</t>
+          <t>Traced (v5.6): legacy process emissions = 2023 inventory x the year-on-year growth of industrial energy CO2 (row 6576; 2024: +16.8%, the rebound after the 2023 demand shock, so 56.9 -&gt; 66.5). The prototype floored that growth at 0 (a departure: removed in v5.6, as legacy). The remaining gap is the industrial energy CO2 path, part of the fuel-use gap (I14).</t>
         </is>
       </c>
       <c r="J154" s="9" t="inlineStr">
@@ -9403,6 +10084,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L154" s="9" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="9" t="inlineStr">
@@ -9443,7 +10125,7 @@
       <c r="H155" s="9" t="inlineStr"/>
       <c r="I155" s="9" t="inlineStr">
         <is>
-          <t>Checked (v5.6): energy N2O moves with energy CO2 as legacy (row 7563 = previous x CO2 ratio). Production for fuel-supply methane differs: now issue I66.</t>
+          <t>Checked (v5.6): energy N2O moves with energy CO2 as legacy (row 7549 = previous x CO2 ratio). Production for fuel-supply methane differs: now issue I66.</t>
         </is>
       </c>
       <c r="J155" s="9" t="inlineStr">
@@ -9456,6 +10138,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L155" s="9" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="9" t="inlineStr">
@@ -9509,6 +10192,7 @@
           <t>Dropped</t>
         </is>
       </c>
+      <c r="L156" s="9" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="9" t="inlineStr">
@@ -9562,6 +10246,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L157" s="9" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="9" t="inlineStr">
@@ -9596,7 +10281,7 @@
       </c>
       <c r="G158" s="9" t="inlineStr">
         <is>
-          <t>Legacy row 7534 ("Adjust EFs to match energy-related CO2 to UNFCCC inventories?", Yes* by default) multiplies every CO2 EF by the inventory energy CO2 of the year before the base year over the estimate from the base-year energy balance (Egypt: 2021 inventory against 2022, 0.930), so CO2 is about 7% below uncalibrated EFs in every sector. The inventory has a break between 2021 and 2022 (I17: 211 to 252 Mt), which legacy carries into the factor. v4.11 replicates legacy (user 2026-10-18: go with legacy); before, the prototype calibrated in 2024 and kept the switch off (user decisions v3.2, v3.4).</t>
+          <t>Legacy row 7520 ("Adjust EFs to match energy-related CO2 to UNFCCC inventories?", Yes* by default) multiplies every CO2 EF by the inventory energy CO2 of the year before the base year over the estimate from the base-year energy balance (Egypt: 2021 inventory against 2022, 0.930), so CO2 is about 7% below uncalibrated EFs in every sector. The inventory has a break between 2021 and 2022 (I17: 211 to 252 Mt), which legacy carries into the factor. v4.11 replicates legacy (user 2026-10-18: go with legacy); before, the prototype calibrated in 2024 and kept the switch off (user decisions v3.2, v3.4).</t>
         </is>
       </c>
       <c r="H158" s="9" t="inlineStr"/>
@@ -9615,6 +10300,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L158" s="9" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="9" t="inlineStr">
@@ -9649,7 +10335,7 @@
       </c>
       <c r="G159" s="9" t="inlineStr">
         <is>
-          <t>Legacy rows 7297-7321 feed the air-pollution module CH4 by sector: oil and gas extraction methane under "other", agriculture and waste methane under "food &amp; forestry" (waste is not food or forestry), no combustion CH4 (no factors in legacy). v3.12 replicates the allocation and adds the combustion CH4 of each sector (GAINS factors, section 14), with all fossil fuel supply methane (extraction, downstream gas, coal mining, biomass) under "other".</t>
+          <t>Legacy rows 7283-7307 feed the air-pollution module CH4 by sector: oil and gas extraction methane under "other", agriculture and waste methane under "food &amp; forestry" (waste is not food or forestry), no combustion CH4 (no factors in legacy). v3.12 replicates the allocation and adds the combustion CH4 of each sector (GAINS factors, section 14), with all fossil fuel supply methane (extraction, downstream gas, coal mining, biomass) under "other".</t>
         </is>
       </c>
       <c r="H159" s="9" t="inlineStr"/>
@@ -9668,6 +10354,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L159" s="9" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="9" t="inlineStr">
@@ -9702,7 +10389,7 @@
       </c>
       <c r="G160" s="9" t="inlineStr">
         <is>
-          <t>Legacy's effective carbon rate (row 16662) and total carbon price (F5d) divide revenue net of subsidies, VAT included, by CO2; the OECD effective carbon rate counts carbon taxes, fuel excises and permit prices only. The prototype replicates the legacy definition (section 17, v3.15) and says so in the note; Egypt has negative rates (subsidies exceed taxes).</t>
+          <t>Legacy's effective carbon rate (row 16647) and total carbon price (F5d) divide revenue net of subsidies, VAT included, by CO2; the OECD effective carbon rate counts carbon taxes, fuel excises and permit prices only. The prototype replicates the legacy definition (section 17, v3.15) and says so in the note; Egypt has negative rates (subsidies exceed taxes).</t>
         </is>
       </c>
       <c r="H160" s="9" t="inlineStr"/>
@@ -9721,6 +10408,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L160" s="9" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="9" t="inlineStr">
@@ -9774,6 +10462,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L161" s="9" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="9" t="inlineStr">
@@ -9827,6 +10516,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L162" s="9" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="9" t="inlineStr">
@@ -9880,6 +10570,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L163" s="9" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="9" t="inlineStr">
@@ -9933,6 +10624,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L164" s="9" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="9" t="inlineStr">
@@ -9967,7 +10659,7 @@
       </c>
       <c r="G165" s="9" t="inlineStr">
         <is>
-          <t>Legacy row 14356 takes the yearly change of the revenue gain in USD over the current GDP, not the change of the gain as a share of GDP: with GDP growing, a constant share of GDP keeps giving impulses (Egypt: impulses sum to 4.9% of GDP against a final fiscal space of 3.5%). Replicated in v4.15 (user 2026-10-18: replicate legacy, note issues).</t>
+          <t>Legacy row 14341 takes the yearly change of the revenue gain in USD over the current GDP, not the change of the gain as a share of GDP: with GDP growing, a constant share of GDP keeps giving impulses (Egypt: impulses sum to 4.9% of GDP against a final fiscal space of 3.5%). Replicated in v4.15 (user 2026-10-18: replicate legacy, note issues).</t>
         </is>
       </c>
       <c r="H165" s="9" t="inlineStr"/>
@@ -9986,6 +10678,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L165" s="9" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="9" t="inlineStr">
@@ -10039,6 +10732,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L166" s="9" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="9" t="inlineStr">
@@ -10092,6 +10786,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L167" s="9" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="9" t="inlineStr">
@@ -10145,6 +10840,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L168" s="9" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="9" t="inlineStr">
@@ -10198,6 +10894,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L169" s="9" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="9" t="inlineStr">
@@ -10232,13 +10929,13 @@
       </c>
       <c r="G170" s="9" t="inlineStr">
         <is>
-          <t>Legacy total revenue (row 8026) includes the transport revenues of the engineer road model (customs and VAT on vehicles, feebates, vehicle and charging subsidies, distance tax; rows 7913-7999) and the renewable subsidy cost (from the elasticity power model even where the engineer model is used, rows 7896-7904). The prototype 12e block has both rows at 0 (road engineer revenues parked; no renewable subsidy policy). Egypt: transport +0.04 bn in 2030 against baseline.</t>
+          <t>Legacy total revenue (row 8012) includes the transport revenues of the engineer road model (customs and VAT on vehicles, feebates, vehicle and charging subsidies, distance tax; rows 7899-7985) and the renewable subsidy cost (from the elasticity power model even where the engineer model is used, rows 7882-7890). The prototype 12e block has both rows at 0 (road engineer revenues parked; no renewable subsidy policy). Egypt: transport +0.04 bn in 2030 against baseline.</t>
         </is>
       </c>
       <c r="H170" s="9" t="inlineStr"/>
       <c r="I170" s="9" t="inlineStr">
         <is>
-          <t>Renewable subsidies: in the power model since v5.4 (prrns), counted in rsub, rtot and block 12e row rpol.ren, as legacy rows 7896-7904. Transport revenues: dropped with the engineer road model (I61, user 2026-10-20); row rpol.trs stays 0.</t>
+          <t>Renewable subsidies: in the power model since v5.4 (prrns), counted in rsub, rtot and block 12e row rpol.ren, as legacy rows 7882-7890. Transport revenues: dropped with the engineer road model (I61, user 2026-10-20); row rpol.trs stays 0.</t>
         </is>
       </c>
       <c r="J170" s="9" t="inlineStr">
@@ -10251,6 +10948,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L170" s="9" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="9" t="inlineStr">
@@ -10304,6 +11002,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L171" s="9" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="9" t="inlineStr">
@@ -10357,6 +11056,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L172" s="9" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="9" t="inlineStr">
@@ -10410,6 +11110,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L173" s="9" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="9" t="inlineStr">
@@ -10463,6 +11164,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L174" s="9" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="9" t="inlineStr">
@@ -10516,6 +11218,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L175" s="9" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="9" t="inlineStr">
@@ -10550,7 +11253,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>MTInputs 354-355 are labelled $/kWh nominal and enter the real cost and revenue without deflation (Mitigation row 2743). Replicated (rows rnsp, rns).</t>
+          <t>MTInputs 352-353 are labelled $/kWh nominal and enter the real cost and revenue without deflation (Mitigation row 2743). Replicated (rows rnsp, rns).</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr"/>
@@ -10569,6 +11272,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L176" s="9" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="9" t="inlineStr">
@@ -10622,6 +11326,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L177" s="9" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="9" t="inlineStr">
@@ -10675,6 +11380,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L178" s="9" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="9" t="inlineStr">
@@ -10728,6 +11434,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L179" s="9" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="9" t="inlineStr">
@@ -10781,6 +11488,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L180" s="9" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="9" t="inlineStr">
@@ -10834,6 +11542,7 @@
           <t>Dropped</t>
         </is>
       </c>
+      <c r="L181" s="9" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="9" t="inlineStr">
@@ -10887,6 +11596,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L182" s="9" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="9" t="inlineStr">
@@ -10940,6 +11650,7 @@
           <t>Dropped</t>
         </is>
       </c>
+      <c r="L183" s="9" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="9" t="inlineStr">
@@ -10974,7 +11685,7 @@
       </c>
       <c r="G184" s="9" t="inlineStr">
         <is>
-          <t>Legacy grows crude oil, natural gas and coal production (rows 6146-6149) from 2024 with the producer-price response to the methane fee (rows 6137-6144: price increase x pass-through, Manual inputs J190:J194 elasticities) and the growth of world demand of the global demand scenario (Prices_int rows 323-333, lagged one year). The prototype holds production at the base year (rows ch4.act og, cm). Found 2026-10-19 checking I26.</t>
+          <t>Legacy grows crude oil, natural gas and coal production (rows 6132-6135) from 2024 with the producer-price response to the methane fee (rows 6123-6130: price increase x pass-through, Manual inputs J190:J194 elasticities) and the growth of world demand of the global demand scenario (Prices_int rows 323-333, lagged one year). The prototype holds production at the base year (rows ch4.act og, cm). Found 2026-10-19 checking I26.</t>
         </is>
       </c>
       <c r="H184" s="9" t="inlineStr"/>
@@ -10993,6 +11704,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L184" s="9" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="9" t="inlineStr">
@@ -11046,6 +11758,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L185" s="9" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="9" t="inlineStr">
@@ -11099,6 +11812,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L186" s="9" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="9" t="inlineStr">
@@ -11133,7 +11847,7 @@
       </c>
       <c r="G187" s="9" t="inlineStr">
         <is>
-          <t>Legacy and the prototype let revenue of year t move GDP only from year t+1 (legacy row 8776 reads the previous column; prototype gdp.lvl = 1 + last year's gdp.eff), and the fiscal space reads revenue of year t only. This lag is what keeps the model free of circular references whatever the revenue lines read; it is not stated anywhere. Recommendation to the CPAT team: make it an explicit rule of the method and keep it when the GDP block changes. Replicated.</t>
+          <t>Legacy and the prototype let revenue of year t move GDP only from year t+1 (legacy row 8761 reads the previous column; prototype gdp.lvl = 1 + last year's gdp.eff), and the fiscal space reads revenue of year t only. This lag is what keeps the model free of circular references whatever the revenue lines read; it is not stated anywhere. Recommendation to the CPAT team: make it an explicit rule of the method and keep it when the GDP block changes. Replicated.</t>
         </is>
       </c>
       <c r="H187" s="9" t="inlineStr"/>
@@ -11152,6 +11866,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L187" s="9" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="9" t="inlineStr">
@@ -11201,6 +11916,7 @@
         </is>
       </c>
       <c r="K188" s="9" t="inlineStr"/>
+      <c r="L188" s="9" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="9" t="inlineStr">
@@ -11250,6 +11966,7 @@
         </is>
       </c>
       <c r="K189" s="9" t="inlineStr"/>
+      <c r="L189" s="9" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="9" t="inlineStr">
@@ -11299,6 +12016,7 @@
         </is>
       </c>
       <c r="K190" s="9" t="inlineStr"/>
+      <c r="L190" s="9" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="9" t="inlineStr">
@@ -11348,6 +12066,7 @@
         </is>
       </c>
       <c r="K191" s="9" t="inlineStr"/>
+      <c r="L191" s="9" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="9" t="inlineStr">
@@ -11397,6 +12116,7 @@
         </is>
       </c>
       <c r="K192" s="9" t="inlineStr"/>
+      <c r="L192" s="9" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="9" t="inlineStr">
@@ -11446,6 +12166,7 @@
         </is>
       </c>
       <c r="K193" s="9" t="inlineStr"/>
+      <c r="L193" s="9" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="9" t="inlineStr">
@@ -11495,6 +12216,7 @@
         </is>
       </c>
       <c r="K194" s="9" t="inlineStr"/>
+      <c r="L194" s="9" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="9" t="inlineStr">
@@ -11544,6 +12266,7 @@
         </is>
       </c>
       <c r="K195" s="9" t="inlineStr"/>
+      <c r="L195" s="9" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="9" t="inlineStr">
@@ -11593,6 +12316,7 @@
         </is>
       </c>
       <c r="K196" s="9" t="inlineStr"/>
+      <c r="L196" s="9" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="9" t="inlineStr">
@@ -11642,6 +12366,7 @@
         </is>
       </c>
       <c r="K197" s="9" t="inlineStr"/>
+      <c r="L197" s="9" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="9" t="inlineStr">
@@ -11691,6 +12416,7 @@
         </is>
       </c>
       <c r="K198" s="9" t="inlineStr"/>
+      <c r="L198" s="9" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="9" t="inlineStr">
@@ -11740,6 +12466,7 @@
         </is>
       </c>
       <c r="K199" s="9" t="inlineStr"/>
+      <c r="L199" s="9" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="9" t="inlineStr">
@@ -11789,6 +12516,7 @@
         </is>
       </c>
       <c r="K200" s="9" t="inlineStr"/>
+      <c r="L200" s="9" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="9" t="inlineStr">
@@ -11838,6 +12566,7 @@
         </is>
       </c>
       <c r="K201" s="9" t="inlineStr"/>
+      <c r="L201" s="9" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="9" t="inlineStr">
@@ -11887,6 +12616,7 @@
         </is>
       </c>
       <c r="K202" s="9" t="inlineStr"/>
+      <c r="L202" s="9" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="9" t="inlineStr">
@@ -11936,6 +12666,7 @@
         </is>
       </c>
       <c r="K203" s="9" t="inlineStr"/>
+      <c r="L203" s="9" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="9" t="inlineStr">
@@ -11985,6 +12716,7 @@
         </is>
       </c>
       <c r="K204" s="9" t="inlineStr"/>
+      <c r="L204" s="9" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="9" t="inlineStr">
@@ -12034,6 +12766,7 @@
         </is>
       </c>
       <c r="K205" s="9" t="inlineStr"/>
+      <c r="L205" s="9" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="9" t="inlineStr">
@@ -12083,6 +12816,7 @@
         </is>
       </c>
       <c r="K206" s="9" t="inlineStr"/>
+      <c r="L206" s="9" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="9" t="inlineStr">
@@ -12132,6 +12866,7 @@
         </is>
       </c>
       <c r="K207" s="9" t="inlineStr"/>
+      <c r="L207" s="9" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="9" t="inlineStr">
@@ -12181,6 +12916,7 @@
         </is>
       </c>
       <c r="K208" s="9" t="inlineStr"/>
+      <c r="L208" s="9" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="9" t="inlineStr">
@@ -12230,6 +12966,7 @@
         </is>
       </c>
       <c r="K209" s="9" t="inlineStr"/>
+      <c r="L209" s="9" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="9" t="inlineStr">
@@ -12279,6 +13016,7 @@
         </is>
       </c>
       <c r="K210" s="9" t="inlineStr"/>
+      <c r="L210" s="9" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="9" t="inlineStr">
@@ -12328,6 +13066,7 @@
         </is>
       </c>
       <c r="K211" s="9" t="inlineStr"/>
+      <c r="L211" s="9" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="9" t="inlineStr">
@@ -12377,6 +13116,7 @@
         </is>
       </c>
       <c r="K212" s="9" t="inlineStr"/>
+      <c r="L212" s="9" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="9" t="inlineStr">
@@ -12430,6 +13170,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L213" s="9" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="9" t="inlineStr">
@@ -12479,6 +13220,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L214" s="9" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="9" t="inlineStr">
@@ -12528,6 +13270,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L215" s="9" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="9" t="inlineStr">
@@ -12577,6 +13320,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L216" s="9" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="9" t="inlineStr">
@@ -12626,6 +13370,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L217" s="9" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="9" t="inlineStr">
@@ -12675,6 +13420,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L218" s="9" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="9" t="inlineStr">
@@ -12724,6 +13470,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L219" s="9" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="9" t="inlineStr">
@@ -12773,6 +13520,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L220" s="9" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="9" t="inlineStr">
@@ -12826,6 +13574,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L221" s="9" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="9" t="inlineStr">
@@ -12875,6 +13624,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L222" s="9" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="9" t="inlineStr">
@@ -12924,6 +13674,7 @@
           <t>Accepted</t>
         </is>
       </c>
+      <c r="L223" s="9" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="9" t="inlineStr">
@@ -12977,6 +13728,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L224" s="9" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="9" t="inlineStr">
@@ -13030,6 +13782,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L225" s="9" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="9" t="inlineStr">
@@ -13083,6 +13836,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L226" s="9" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="9" t="inlineStr">
@@ -13136,6 +13890,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L227" s="9" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="9" t="inlineStr">
@@ -13176,7 +13931,7 @@
       <c r="H228" s="9" t="inlineStr"/>
       <c r="I228" s="9" t="inlineStr">
         <is>
-          <t>Legacy checked: no bug. The source allocation uses energy-balance data (row 894) and the energy CH4 calibration (row 7562) uses the first two years and applies the factor from the third (it reads only earlier years). The prototype calibrated on GHGYear (2024) in every year (its own design) and now reads stored scenario-1 values; the fiscal space uses the stored scenario-1 activity (I47).</t>
+          <t>Legacy checked: no bug. The source allocation uses energy-balance data (row 894) and the energy CH4 calibration (row 7548) uses the first two years and applies the factor from the third (it reads only earlier years). The prototype calibrated on GHGYear (2024) in every year (its own design) and now reads stored scenario-1 values; the fiscal space uses the stored scenario-1 activity (I47).</t>
         </is>
       </c>
       <c r="J228" s="9" t="inlineStr">
@@ -13189,6 +13944,7 @@
           <t>Resolved</t>
         </is>
       </c>
+      <c r="L228" s="9" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="9" t="inlineStr">
@@ -13242,6 +13998,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L229" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="9" t="inlineStr">
@@ -13295,6 +14056,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L230" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="9" t="inlineStr">
@@ -13348,6 +14114,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L231" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="9" t="inlineStr">
@@ -13401,6 +14172,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L232" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="9" t="inlineStr">
@@ -13454,6 +14230,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L233" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="9" t="inlineStr">
@@ -13507,6 +14288,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L234" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="9" t="inlineStr">
@@ -13560,6 +14346,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L235" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="9" t="inlineStr">
@@ -13613,6 +14404,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L236" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="9" t="inlineStr">
@@ -13666,6 +14462,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L237" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="9" t="inlineStr">
@@ -13719,6 +14520,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L238" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="9" t="inlineStr">
@@ -13772,6 +14578,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L239" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="9" t="inlineStr">
@@ -13825,6 +14636,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L240" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="9" t="inlineStr">
@@ -13878,6 +14694,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L241" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="9" t="inlineStr">
@@ -13931,6 +14752,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L242" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="9" t="inlineStr">
@@ -13984,6 +14810,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L243" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="9" t="inlineStr">
@@ -14037,6 +14868,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L244" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="9" t="inlineStr">
@@ -14090,6 +14926,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L245" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="9" t="inlineStr">
@@ -14143,6 +14984,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L246" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="9" t="inlineStr">
@@ -14196,6 +15042,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L247" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="9" t="inlineStr">
@@ -14249,6 +15100,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L248" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="9" t="inlineStr">
@@ -14302,6 +15158,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L249" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="9" t="inlineStr">
@@ -14355,6 +15216,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L250" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="9" t="inlineStr">
@@ -14408,6 +15274,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L251" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="9" t="inlineStr">
@@ -14461,6 +15332,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L252" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="9" t="inlineStr">
@@ -14514,6 +15390,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L253" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="9" t="inlineStr">
@@ -14567,6 +15448,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L254" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="9" t="inlineStr">
@@ -14620,6 +15506,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L255" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="9" t="inlineStr">
@@ -14673,6 +15564,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L256" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="9" t="inlineStr">
@@ -14726,6 +15622,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L257" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="9" t="inlineStr">
@@ -14779,6 +15680,11 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L258" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="9" t="inlineStr">
@@ -14830,6 +15736,11 @@
       <c r="K259" s="9" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="L259" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -14877,6 +15788,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L260" s="9" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" s="9" t="inlineStr">
@@ -14922,6 +15834,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L261" s="9" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" s="9" t="inlineStr">
@@ -14967,6 +15880,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L262" s="9" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="9" t="inlineStr">
@@ -15012,6 +15926,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L263" s="9" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="9" t="inlineStr">
@@ -15057,6 +15972,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L264" s="9" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" s="9" t="inlineStr">
@@ -15102,6 +16018,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L265" s="9" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="9" t="inlineStr">
@@ -15147,6 +16064,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L266" s="9" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="9" t="inlineStr">
@@ -15192,6 +16110,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L267" s="9" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="9" t="inlineStr">
@@ -15237,6 +16156,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L268" s="9" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" s="9" t="inlineStr">
@@ -15282,6 +16202,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="L269" s="9" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" s="9" t="inlineStr">
@@ -15331,6 +16252,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L270" s="9" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" s="9" t="inlineStr">
@@ -15380,6 +16302,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L271" s="9" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" s="9" t="inlineStr">
@@ -15429,6 +16352,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L272" s="9" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" s="9" t="inlineStr">
@@ -15478,6 +16402,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L273" s="9" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" s="9" t="inlineStr">
@@ -15527,6 +16452,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L274" s="9" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" s="9" t="inlineStr">
@@ -15576,6 +16502,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L275" s="9" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" s="9" t="inlineStr">
@@ -15625,6 +16552,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L276" s="9" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" s="9" t="inlineStr">
@@ -15674,6 +16602,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L277" s="9" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" s="9" t="inlineStr">
@@ -15723,6 +16652,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L278" s="9" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" s="9" t="inlineStr">
@@ -15772,6 +16702,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L279" s="9" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" s="9" t="inlineStr">
@@ -15821,6 +16752,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L280" s="9" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" s="9" t="inlineStr">
@@ -15870,6 +16802,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L281" s="9" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" s="9" t="inlineStr">
@@ -15919,6 +16852,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L282" s="9" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" s="9" t="inlineStr">
@@ -15968,9 +16902,10 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="L283" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K283"/>
+  <autoFilter ref="A3:L283"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>